<commit_message>
Extract core topic keywords and save to new excel file format
</commit_message>
<xml_diff>
--- a/타기관벤치마킹_20260807.xlsx
+++ b/타기관벤치마킹_20260807.xlsx
@@ -455,14 +455,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="65" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -478,15 +479,20 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>매칭키워드</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>등록일</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>마감일</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>링크</t>
         </is>
@@ -505,15 +511,20 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t>창업기업 모집공고</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>https://www.mss.go.kr/site/smba/ex/bbs/View.do?cbIdx=310&amp;bcIdx=1070326</t>
         </is>
@@ -527,21 +538,25 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>[공고]
-											2026년 외국인근로자 주거환경개선 지원 보조사업자 선정 결과 공고</t>
+          <t>[공고] 2026년 외국인근로자 주거환경개선 지원 보조사업자 선정 결과 공고</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
+          <t>보조사업자 선정 결과</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>2026-08-05</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>https://www.moel.go.kr/news/notice/noticeView.do?bbs_seq=20260800173</t>
         </is>
@@ -560,15 +575,20 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
+          <t>참여기업 모집공고</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>https://www.mss.go.kr/site/smba/ex/bbs/View.do?cbIdx=310&amp;bcIdx=1070215</t>
         </is>
@@ -582,21 +602,25 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>[공고]
-											일반임기제 행정5급(사회적금융 정책 지원) 공무원 경력경쟁채용시험 공고</t>
+          <t>[공고] 일반임기제 행정5급(사회적금융 정책 지원) 공무원 경력경쟁채용시험 공고</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
+          <t>경력채용시험 공고</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>https://www.moel.go.kr/news/notice/noticeView.do?bbs_seq=20260800030</t>
         </is>
@@ -615,17 +639,22 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
+          <t>합격자 공고</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=G7UvOsRZBhs5s6d6JQIacNb-NezWJrPj9W05sDmM.node30?bbsId=BBSMSTR_000000000006&amp;nttId=128313</t>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=-_zzglc5PwMahzKGEZeZU68tewg7AnOGOZf210ba.node30?bbsId=BBSMSTR_000000000006&amp;nttId=128313</t>
         </is>
       </c>
     </row>
@@ -637,21 +666,25 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>[공고]
-											고용노동부 민원 처리 담당자 보호 및 지원에 관한 규정 제정(안) 행정예고</t>
+          <t>[공고] 고용노동부 민원 처리 담당자 보호 및 지원에 관한 규정 제정(안) 행정예고</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
+          <t>규정 제정 행정예고</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>https://www.moel.go.kr/news/notice/noticeView.do?bbs_seq=20260701070</t>
         </is>
@@ -670,17 +703,22 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
+          <t>신규 지정 공모</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=npf6QW5PzwHy40oUUrBNqYyvvxUUrieu3qTFu6G-.node10?bbsId=BBSMSTR_000000000006&amp;nttId=128214</t>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=Ks2YxHDrOfIGHbR6cWMKCcyiZvcf3XOpxP_TzQAg.node50?bbsId=BBSMSTR_000000000006&amp;nttId=128214</t>
         </is>
       </c>
     </row>
@@ -697,17 +735,22 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
+          <t>경력채용시험 공고</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=g-F2EZwTnBiQLkOBnA1owwme7U26xcte8I_p_flC.node30?bbsId=BBSMSTR_000000000006&amp;nttId=128199</t>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=31cKibTqiRqVEXnWlYlG79-4QlhgKwi-3ttsJqKp.node10?bbsId=BBSMSTR_000000000006&amp;nttId=128199</t>
         </is>
       </c>
     </row>
@@ -724,17 +767,22 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
+          <t>포상 후보자 공모</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=g-F2EZwTnBiQLkOBnA1owwme7U26xcte8I_p_flC.node30?bbsId=BBSMSTR_000000000006&amp;nttId=128194</t>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=31cKibTqiRqVEXnWlYlG79-4QlhgKwi-3ttsJqKp.node10?bbsId=BBSMSTR_000000000006&amp;nttId=128194</t>
         </is>
       </c>
     </row>
@@ -751,15 +799,20 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
+          <t>창업기업 모집공고</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>https://www.mss.go.kr/site/smba/ex/bbs/View.do?cbIdx=310&amp;bcIdx=1070051</t>
         </is>
@@ -773,21 +826,25 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>[공고]
-											제5회 고용노동 공공데이터·AI 활용 공모전 수상작 선정 결과</t>
+          <t>[공고] 제5회 고용노동 공공데이터·AI 활용 공모전 수상작 선정 결과</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
+          <t>공모전 수상작 선정 결과</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
           <t>2026-07-22</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>https://www.moel.go.kr/news/notice/noticeView.do?bbs_seq=20260700774</t>
         </is>
@@ -806,17 +863,22 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
+          <t>기술능력평가 결과 알림</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
           <t>2026-07-21</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=3IubyDrOHYj-ZThMaYXasUq5ySYg2Ij18t6eX_W9.node50?bbsId=BBSMSTR_000000000006&amp;nttId=128068</t>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=aZQ9Cla2dsZ0Ybzl-29ZeusCNix_2JY897dXlzzc.node20?bbsId=BBSMSTR_000000000006&amp;nttId=128068</t>
         </is>
       </c>
     </row>
@@ -833,17 +895,22 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
+          <t>교육기관 선정 공고</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
           <t>2026-07-21</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=j-gXDBHUaeBCy32YPE3vwLXPTKYhIpN5J2hRWCht.node10?bbsId=BBSMSTR_000000000006&amp;nttId=128057</t>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=9JLumN8jLuW-7uzbSaFEKAbOcQy1P5Qyxj_85NIt.node10?bbsId=BBSMSTR_000000000006&amp;nttId=128057</t>
         </is>
       </c>
     </row>
@@ -860,15 +927,20 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
+          <t>지원사업 공고</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
           <t>2026-07-20</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>https://www.mss.go.kr/site/smba/ex/bbs/View.do?cbIdx=310&amp;bcIdx=1069923</t>
         </is>
@@ -887,15 +959,20 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
+          <t>참여기업 모집공고</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>https://www.mss.go.kr/site/smba/ex/bbs/View.do?cbIdx=310&amp;bcIdx=1069894</t>
         </is>
@@ -914,15 +991,20 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
+          <t>창업기업 모집공고</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>https://www.mss.go.kr/site/smba/ex/bbs/View.do?cbIdx=310&amp;bcIdx=1069892</t>
         </is>
@@ -941,15 +1023,20 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
+          <t>참여기업 모집공고</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>https://www.mss.go.kr/site/smba/ex/bbs/View.do?cbIdx=310&amp;bcIdx=1069829</t>
         </is>
@@ -968,17 +1055,22 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
+          <t>경력채용시험 공고</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=j-gXDBHUaeBCy32YPE3vwLXPTKYhIpN5J2hRWCht.node10?bbsId=BBSMSTR_000000000006&amp;nttId=127882</t>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=9JLumN8jLuW-7uzbSaFEKAbOcQy1P5Qyxj_85NIt.node10?bbsId=BBSMSTR_000000000006&amp;nttId=127882</t>
         </is>
       </c>
     </row>
@@ -990,21 +1082,25 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>[인사]
-											고용노동부 공모 직위(고용지원실업급여과장) 공개모집(연장)</t>
+          <t>[인사] 고용노동부 공모 직위(고용지원실업급여과장) 공개모집(연장)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
+          <t>직위 공개모집</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>https://www.moel.go.kr/news/notice/noticeView.do?bbs_seq=20260700508</t>
         </is>
@@ -1023,17 +1119,22 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
+          <t>창업경진대회 공고</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=2OZsrK7u0fCFF-K90H8On0mh17An9jPLhCEdThPb.node30?bbsId=BBSMSTR_000000000006&amp;nttId=127805</t>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=Rm-cLaO5_M_-74BPp-LKtrl89JgRRgGrjg9Ef5ET.node10?bbsId=BBSMSTR_000000000006&amp;nttId=127805</t>
         </is>
       </c>
     </row>
@@ -1050,15 +1151,20 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
+          <t>지원계획 공고</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>https://www.mss.go.kr/site/smba/ex/bbs/View.do?cbIdx=310&amp;bcIdx=1069726</t>
         </is>
@@ -1077,15 +1183,20 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
+          <t>창업기업 모집공고</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>https://www.mss.go.kr/site/smba/ex/bbs/View.do?cbIdx=310&amp;bcIdx=1069709</t>
         </is>
@@ -1099,21 +1210,25 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>[공고]
-											근로복지공단 이사장 공개 모집</t>
+          <t>[공고] 근로복지공단 이사장 공개 모집</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
+          <t>근로복지공단 이사장 공개 모집</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>https://www.moel.go.kr/news/notice/noticeView.do?bbs_seq=20260700360</t>
         </is>
@@ -1132,15 +1247,20 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
+          <t>참여기업 모집공고</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>https://www.mss.go.kr/site/smba/ex/bbs/View.do?cbIdx=310&amp;bcIdx=1069686</t>
         </is>
@@ -1157,14 +1277,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="65" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1180,15 +1301,20 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>매칭키워드</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>등록일</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>마감일</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>링크</t>
         </is>
@@ -1207,17 +1333,22 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t>합격자 공고</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=G7UvOsRZBhs5s6d6JQIacNb-NezWJrPj9W05sDmM.node30?bbsId=BBSMSTR_000000000006&amp;nttId=128313</t>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=-_zzglc5PwMahzKGEZeZU68tewg7AnOGOZf210ba.node30?bbsId=BBSMSTR_000000000006&amp;nttId=128313</t>
         </is>
       </c>
     </row>
@@ -1234,17 +1365,22 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
+          <t>신규 지정 공모</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=npf6QW5PzwHy40oUUrBNqYyvvxUUrieu3qTFu6G-.node10?bbsId=BBSMSTR_000000000006&amp;nttId=128214</t>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=Ks2YxHDrOfIGHbR6cWMKCcyiZvcf3XOpxP_TzQAg.node50?bbsId=BBSMSTR_000000000006&amp;nttId=128214</t>
         </is>
       </c>
     </row>
@@ -1261,17 +1397,22 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
+          <t>경력채용시험 공고</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=g-F2EZwTnBiQLkOBnA1owwme7U26xcte8I_p_flC.node30?bbsId=BBSMSTR_000000000006&amp;nttId=128199</t>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=31cKibTqiRqVEXnWlYlG79-4QlhgKwi-3ttsJqKp.node10?bbsId=BBSMSTR_000000000006&amp;nttId=128199</t>
         </is>
       </c>
     </row>
@@ -1288,17 +1429,22 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
+          <t>포상 후보자 공모</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=g-F2EZwTnBiQLkOBnA1owwme7U26xcte8I_p_flC.node30?bbsId=BBSMSTR_000000000006&amp;nttId=128194</t>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=31cKibTqiRqVEXnWlYlG79-4QlhgKwi-3ttsJqKp.node10?bbsId=BBSMSTR_000000000006&amp;nttId=128194</t>
         </is>
       </c>
     </row>
@@ -1315,17 +1461,22 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
+          <t>기술능력평가 결과 알림</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
           <t>2026-07-21</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=3IubyDrOHYj-ZThMaYXasUq5ySYg2Ij18t6eX_W9.node50?bbsId=BBSMSTR_000000000006&amp;nttId=128068</t>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=aZQ9Cla2dsZ0Ybzl-29ZeusCNix_2JY897dXlzzc.node20?bbsId=BBSMSTR_000000000006&amp;nttId=128068</t>
         </is>
       </c>
     </row>
@@ -1342,17 +1493,22 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
+          <t>교육기관 선정 공고</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
           <t>2026-07-21</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=j-gXDBHUaeBCy32YPE3vwLXPTKYhIpN5J2hRWCht.node10?bbsId=BBSMSTR_000000000006&amp;nttId=128057</t>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=9JLumN8jLuW-7uzbSaFEKAbOcQy1P5Qyxj_85NIt.node10?bbsId=BBSMSTR_000000000006&amp;nttId=128057</t>
         </is>
       </c>
     </row>
@@ -1369,17 +1525,22 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
+          <t>경력채용시험 공고</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=j-gXDBHUaeBCy32YPE3vwLXPTKYhIpN5J2hRWCht.node10?bbsId=BBSMSTR_000000000006&amp;nttId=127882</t>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=9JLumN8jLuW-7uzbSaFEKAbOcQy1P5Qyxj_85NIt.node10?bbsId=BBSMSTR_000000000006&amp;nttId=127882</t>
         </is>
       </c>
     </row>
@@ -1396,17 +1557,22 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
+          <t>창업경진대회 공고</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=2OZsrK7u0fCFF-K90H8On0mh17An9jPLhCEdThPb.node30?bbsId=BBSMSTR_000000000006&amp;nttId=127805</t>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mois.go.kr/frt/bbs/type013/commonSelectBoardArticle.do;jsessionid=Rm-cLaO5_M_-74BPp-LKtrl89JgRRgGrjg9Ef5ET.node10?bbsId=BBSMSTR_000000000006&amp;nttId=127805</t>
         </is>
       </c>
     </row>
@@ -1421,14 +1587,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="65" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1444,15 +1611,20 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>매칭키워드</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>등록일</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>마감일</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>링크</t>
         </is>
@@ -1471,15 +1643,20 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t>창업기업 모집공고</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>https://www.mss.go.kr/site/smba/ex/bbs/View.do?cbIdx=310&amp;bcIdx=1070326</t>
         </is>
@@ -1498,15 +1675,20 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
+          <t>참여기업 모집공고</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>https://www.mss.go.kr/site/smba/ex/bbs/View.do?cbIdx=310&amp;bcIdx=1070215</t>
         </is>
@@ -1525,15 +1707,20 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
+          <t>창업기업 모집공고</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>https://www.mss.go.kr/site/smba/ex/bbs/View.do?cbIdx=310&amp;bcIdx=1070051</t>
         </is>
@@ -1552,15 +1739,20 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
+          <t>지원사업 공고</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
           <t>2026-07-20</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>https://www.mss.go.kr/site/smba/ex/bbs/View.do?cbIdx=310&amp;bcIdx=1069923</t>
         </is>
@@ -1579,15 +1771,20 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
+          <t>참여기업 모집공고</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>https://www.mss.go.kr/site/smba/ex/bbs/View.do?cbIdx=310&amp;bcIdx=1069894</t>
         </is>
@@ -1606,15 +1803,20 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
+          <t>창업기업 모집공고</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>https://www.mss.go.kr/site/smba/ex/bbs/View.do?cbIdx=310&amp;bcIdx=1069892</t>
         </is>
@@ -1633,15 +1835,20 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
+          <t>참여기업 모집공고</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>https://www.mss.go.kr/site/smba/ex/bbs/View.do?cbIdx=310&amp;bcIdx=1069829</t>
         </is>
@@ -1660,15 +1867,20 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
+          <t>지원계획 공고</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>https://www.mss.go.kr/site/smba/ex/bbs/View.do?cbIdx=310&amp;bcIdx=1069726</t>
         </is>
@@ -1687,15 +1899,20 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
+          <t>창업기업 모집공고</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>https://www.mss.go.kr/site/smba/ex/bbs/View.do?cbIdx=310&amp;bcIdx=1069709</t>
         </is>
@@ -1714,15 +1931,20 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
+          <t>참여기업 모집공고</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>https://www.mss.go.kr/site/smba/ex/bbs/View.do?cbIdx=310&amp;bcIdx=1069686</t>
         </is>
@@ -1739,14 +1961,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="65" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1762,15 +1985,20 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>매칭키워드</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>등록일</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>마감일</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>링크</t>
         </is>
@@ -1784,21 +2012,25 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>[공고]
-											2026년 외국인근로자 주거환경개선 지원 보조사업자 선정 결과 공고</t>
+          <t>[공고] 2026년 외국인근로자 주거환경개선 지원 보조사업자 선정 결과 공고</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t>보조사업자 선정 결과</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
           <t>2026-08-05</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>https://www.moel.go.kr/news/notice/noticeView.do?bbs_seq=20260800173</t>
         </is>
@@ -1812,21 +2044,25 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>[공고]
-											일반임기제 행정5급(사회적금융 정책 지원) 공무원 경력경쟁채용시험 공고</t>
+          <t>[공고] 일반임기제 행정5급(사회적금융 정책 지원) 공무원 경력경쟁채용시험 공고</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
+          <t>경력채용시험 공고</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>https://www.moel.go.kr/news/notice/noticeView.do?bbs_seq=20260800030</t>
         </is>
@@ -1840,21 +2076,25 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>[공고]
-											고용노동부 민원 처리 담당자 보호 및 지원에 관한 규정 제정(안) 행정예고</t>
+          <t>[공고] 고용노동부 민원 처리 담당자 보호 및 지원에 관한 규정 제정(안) 행정예고</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
+          <t>규정 제정 행정예고</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>https://www.moel.go.kr/news/notice/noticeView.do?bbs_seq=20260701070</t>
         </is>
@@ -1868,21 +2108,25 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>[공고]
-											제5회 고용노동 공공데이터·AI 활용 공모전 수상작 선정 결과</t>
+          <t>[공고] 제5회 고용노동 공공데이터·AI 활용 공모전 수상작 선정 결과</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
+          <t>공모전 수상작 선정 결과</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
           <t>2026-07-22</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>https://www.moel.go.kr/news/notice/noticeView.do?bbs_seq=20260700774</t>
         </is>
@@ -1896,21 +2140,25 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>[인사]
-											고용노동부 공모 직위(고용지원실업급여과장) 공개모집(연장)</t>
+          <t>[인사] 고용노동부 공모 직위(고용지원실업급여과장) 공개모집(연장)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
+          <t>직위 공개모집</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>https://www.moel.go.kr/news/notice/noticeView.do?bbs_seq=20260700508</t>
         </is>
@@ -1924,21 +2172,25 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>[공고]
-											근로복지공단 이사장 공개 모집</t>
+          <t>[공고] 근로복지공단 이사장 공개 모집</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
+          <t>근로복지공단 이사장 공개 모집</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>상시/정보없음</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>상시/정보없음</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>https://www.moel.go.kr/news/notice/noticeView.do?bbs_seq=20260700360</t>
         </is>

</xml_diff>